<commit_message>
* init data sql파일 수정: tbl_tenant_config 인서트 쿼리에 config_type 컬럼 추가
</commit_message>
<xml_diff>
--- a/docs/config/tbl_tenant_config 정리문서.xlsx
+++ b/docs/config/tbl_tenant_config 정리문서.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\workspace\ezFlow4Java\docs\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NC383\eGovFrameDev\workspace\ezFlow4Java\docs\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="0" windowWidth="24015" windowHeight="11145"/>
+    <workbookView xWindow="3510" yWindow="0" windowWidth="24015" windowHeight="11145"/>
   </bookViews>
   <sheets>
     <sheet name="tbl_tenant_config" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="624">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="706" uniqueCount="626">
   <si>
     <t>LangPrimary3</t>
   </si>
@@ -2957,13 +2957,19 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>NO</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>USE_COMMUNITY</t>
+  </si>
+  <si>
     <t>YES : 사용
 NO : 사용안함</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>NO</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+    <t>커뮤니티 모듈 사용여부</t>
   </si>
 </sst>
 </file>
@@ -3431,7 +3437,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D188"/>
+  <dimension ref="A1:D189"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40.625" style="2" customWidth="1"/>
@@ -5967,10 +5973,24 @@
         <v>621</v>
       </c>
       <c r="C188" s="19" t="s">
+        <v>624</v>
+      </c>
+      <c r="D188" s="13" t="s">
         <v>622</v>
       </c>
-      <c r="D188" s="13" t="s">
+    </row>
+    <row r="189" spans="1:4" ht="27" x14ac:dyDescent="0.3">
+      <c r="A189" s="20" t="s">
         <v>623</v>
+      </c>
+      <c r="B189" s="18" t="s">
+        <v>625</v>
+      </c>
+      <c r="C189" s="19" t="s">
+        <v>624</v>
+      </c>
+      <c r="D189" s="13" t="s">
+        <v>452</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
* tbl_tenant_config 정리문서 업데이트
</commit_message>
<xml_diff>
--- a/docs/config/tbl_tenant_config 정리문서.xlsx
+++ b/docs/config/tbl_tenant_config 정리문서.xlsx
@@ -3,6 +3,11 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="164011"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DC317\git\ezFlow4Java\docs\config\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="17325" windowHeight="7860"/>
   </bookViews>
@@ -14,7 +19,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">tbl_tenant_config!$A$1:$D$186</definedName>
   </definedNames>
   <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -24,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="714" uniqueCount="631">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="635">
   <si>
     <t>LangPrimary3</t>
   </si>
@@ -2990,6 +2994,23 @@
     <t>loginCookieSSO라는 쿠키에 도메인으로 설정하여 로그인 쿠키 하나 추가로 생성
 NO: 사용안함
 그 외의 값은 쿠키 도메인 값이 됨</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>chkSchedulePublic</t>
+  </si>
+  <si>
+    <t>일정작성시 사용자의 일정 공개 기본값 설정 기능 사용 여부 
+ON : 일정 공개/비공개 기본값 설정 기능 사용
+OFF : 일정 비공개 기본값 설정</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>일정등록 공개범위 기본값 설정 여부</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NO</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -3458,7 +3479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D191"/>
+  <dimension ref="A1:D192"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40.625" style="2" customWidth="1"/>
@@ -4326,7 +4347,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="63" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A63" s="6" t="s">
         <v>99</v>
       </c>
@@ -4340,7 +4361,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="64" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A64" s="6" t="s">
         <v>625</v>
       </c>
@@ -4354,7 +4375,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="65" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A65" s="6" t="s">
         <v>600</v>
       </c>
@@ -4368,7 +4389,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="66" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A66" s="6" t="s">
         <v>100</v>
       </c>
@@ -4382,7 +4403,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="67" spans="1:4" s="2" customFormat="1" ht="54" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:4" ht="54" x14ac:dyDescent="0.3">
       <c r="A67" s="6" t="s">
         <v>343</v>
       </c>
@@ -4396,7 +4417,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="68" spans="1:4" s="2" customFormat="1" ht="54" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:4" ht="54" x14ac:dyDescent="0.3">
       <c r="A68" s="6" t="s">
         <v>344</v>
       </c>
@@ -4410,7 +4431,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="69" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A69" s="6" t="s">
         <v>101</v>
       </c>
@@ -4424,7 +4445,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="70" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A70" s="6" t="s">
         <v>103</v>
       </c>
@@ -4438,7 +4459,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="71" spans="1:4" s="2" customFormat="1" ht="67.5" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" ht="67.5" x14ac:dyDescent="0.3">
       <c r="A71" s="6" t="s">
         <v>105</v>
       </c>
@@ -4452,7 +4473,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="72" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A72" s="6" t="s">
         <v>109</v>
       </c>
@@ -4466,7 +4487,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="73" spans="1:4" s="2" customFormat="1" ht="81" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" ht="81" x14ac:dyDescent="0.3">
       <c r="A73" s="6" t="s">
         <v>387</v>
       </c>
@@ -4480,7 +4501,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="74" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A74" s="6" t="s">
         <v>574</v>
       </c>
@@ -4494,7 +4515,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="75" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A75" s="6" t="s">
         <v>111</v>
       </c>
@@ -4508,7 +4529,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="76" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A76" s="6" t="s">
         <v>113</v>
       </c>
@@ -4522,7 +4543,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="77" spans="1:4" s="2" customFormat="1" ht="94.5" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" ht="94.5" x14ac:dyDescent="0.3">
       <c r="A77" s="6" t="s">
         <v>115</v>
       </c>
@@ -4536,7 +4557,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="78" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A78" s="6" t="s">
         <v>271</v>
       </c>
@@ -4550,7 +4571,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="79" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A79" s="6" t="s">
         <v>273</v>
       </c>
@@ -4564,7 +4585,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="80" spans="1:4" s="2" customFormat="1" ht="67.5" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" ht="67.5" x14ac:dyDescent="0.3">
       <c r="A80" s="6" t="s">
         <v>117</v>
       </c>
@@ -4578,7 +4599,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="81" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A81" s="6" t="s">
         <v>575</v>
       </c>
@@ -4592,7 +4613,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="82" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A82" s="6" t="s">
         <v>121</v>
       </c>
@@ -4606,7 +4627,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="83" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" s="6" t="s">
         <v>275</v>
       </c>
@@ -4620,7 +4641,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="84" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A84" s="6" t="s">
         <v>123</v>
       </c>
@@ -4634,7 +4655,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="85" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A85" s="6" t="s">
         <v>125</v>
       </c>
@@ -4648,7 +4669,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="86" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A86" s="6" t="s">
         <v>576</v>
       </c>
@@ -4662,7 +4683,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="87" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A87" s="6" t="s">
         <v>346</v>
       </c>
@@ -4676,7 +4697,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="88" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A88" s="6" t="s">
         <v>129</v>
       </c>
@@ -4690,7 +4711,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="89" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A89" s="6" t="s">
         <v>128</v>
       </c>
@@ -4704,7 +4725,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="90" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A90" s="6" t="s">
         <v>133</v>
       </c>
@@ -4718,7 +4739,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="91" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A91" s="6" t="s">
         <v>134</v>
       </c>
@@ -4732,7 +4753,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="92" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A92" s="6" t="s">
         <v>135</v>
       </c>
@@ -4746,7 +4767,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="93" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A93" s="6" t="s">
         <v>138</v>
       </c>
@@ -4760,7 +4781,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="94" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A94" s="6" t="s">
         <v>140</v>
       </c>
@@ -4774,7 +4795,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="95" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A95" s="6" t="s">
         <v>143</v>
       </c>
@@ -4788,7 +4809,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="96" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A96" s="6" t="s">
         <v>16</v>
       </c>
@@ -4802,7 +4823,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="97" spans="1:4" s="2" customFormat="1" ht="54" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:4" ht="54" x14ac:dyDescent="0.3">
       <c r="A97" s="6" t="s">
         <v>148</v>
       </c>
@@ -4816,7 +4837,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="98" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A98" s="6" t="s">
         <v>347</v>
       </c>
@@ -4830,7 +4851,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="99" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A99" s="6" t="s">
         <v>350</v>
       </c>
@@ -4844,7 +4865,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="100" spans="1:4" s="2" customFormat="1" ht="54" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:4" ht="54" x14ac:dyDescent="0.3">
       <c r="A100" s="6" t="s">
         <v>17</v>
       </c>
@@ -4858,7 +4879,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="101" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A101" s="6" t="s">
         <v>352</v>
       </c>
@@ -4870,7 +4891,7 @@
       </c>
       <c r="D101" s="13"/>
     </row>
-    <row r="102" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A102" s="6" t="s">
         <v>151</v>
       </c>
@@ -4884,7 +4905,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="103" spans="1:4" s="2" customFormat="1" ht="54" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:4" ht="54" x14ac:dyDescent="0.3">
       <c r="A103" s="6" t="s">
         <v>586</v>
       </c>
@@ -4896,7 +4917,7 @@
       </c>
       <c r="D103" s="13"/>
     </row>
-    <row r="104" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A104" s="6" t="s">
         <v>154</v>
       </c>
@@ -4910,7 +4931,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="105" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A105" s="6" t="s">
         <v>157</v>
       </c>
@@ -4924,7 +4945,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="106" spans="1:4" s="2" customFormat="1" ht="94.5" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:4" ht="94.5" x14ac:dyDescent="0.3">
       <c r="A106" s="6" t="s">
         <v>158</v>
       </c>
@@ -4938,7 +4959,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="107" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A107" s="6" t="s">
         <v>160</v>
       </c>
@@ -4952,7 +4973,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="108" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A108" s="6" t="s">
         <v>304</v>
       </c>
@@ -4964,7 +4985,7 @@
       </c>
       <c r="D108" s="13"/>
     </row>
-    <row r="109" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A109" s="6" t="s">
         <v>278</v>
       </c>
@@ -4976,7 +4997,7 @@
       </c>
       <c r="D109" s="13"/>
     </row>
-    <row r="110" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A110" s="6" t="s">
         <v>356</v>
       </c>
@@ -4990,7 +5011,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="111" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A111" s="6" t="s">
         <v>18</v>
       </c>
@@ -5002,7 +5023,7 @@
       </c>
       <c r="D111" s="13"/>
     </row>
-    <row r="112" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A112" s="6" t="s">
         <v>19</v>
       </c>
@@ -5014,7 +5035,7 @@
       </c>
       <c r="D112" s="13"/>
     </row>
-    <row r="113" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A113" s="6" t="s">
         <v>164</v>
       </c>
@@ -5028,7 +5049,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="114" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A114" s="6" t="s">
         <v>446</v>
       </c>
@@ -5042,7 +5063,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="115" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A115" s="6" t="s">
         <v>165</v>
       </c>
@@ -5056,7 +5077,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="116" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A116" s="6" t="s">
         <v>167</v>
       </c>
@@ -5070,7 +5091,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="117" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A117" s="6" t="s">
         <v>577</v>
       </c>
@@ -5082,7 +5103,7 @@
       </c>
       <c r="D117" s="13"/>
     </row>
-    <row r="118" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A118" s="6" t="s">
         <v>395</v>
       </c>
@@ -5094,7 +5115,7 @@
       </c>
       <c r="D118" s="13"/>
     </row>
-    <row r="119" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A119" s="6" t="s">
         <v>171</v>
       </c>
@@ -5108,7 +5129,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="120" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A120" s="6" t="s">
         <v>390</v>
       </c>
@@ -5122,7 +5143,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="121" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A121" s="6" t="s">
         <v>393</v>
       </c>
@@ -5134,7 +5155,7 @@
       </c>
       <c r="D121" s="13"/>
     </row>
-    <row r="122" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A122" s="6" t="s">
         <v>6</v>
       </c>
@@ -5144,7 +5165,7 @@
       <c r="C122" s="5"/>
       <c r="D122" s="13"/>
     </row>
-    <row r="123" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A123" s="6" t="s">
         <v>5</v>
       </c>
@@ -5156,7 +5177,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="124" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A124" s="6" t="s">
         <v>4</v>
       </c>
@@ -5168,7 +5189,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="125" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A125" s="6" t="s">
         <v>3</v>
       </c>
@@ -5180,7 +5201,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="126" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A126" s="6" t="s">
         <v>412</v>
       </c>
@@ -5194,7 +5215,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="127" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A127" s="6" t="s">
         <v>2</v>
       </c>
@@ -5204,7 +5225,7 @@
       <c r="C127" s="5"/>
       <c r="D127" s="13"/>
     </row>
-    <row r="128" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A128" s="6" t="s">
         <v>1</v>
       </c>
@@ -5216,7 +5237,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="129" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A129" s="6" t="s">
         <v>0</v>
       </c>
@@ -5228,7 +5249,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="130" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A130" s="6" t="s">
         <v>410</v>
       </c>
@@ -5240,7 +5261,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="131" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A131" s="6" t="s">
         <v>578</v>
       </c>
@@ -5254,7 +5275,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="132" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A132" s="6" t="s">
         <v>288</v>
       </c>
@@ -5266,7 +5287,7 @@
       </c>
       <c r="D132" s="13"/>
     </row>
-    <row r="133" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A133" s="6" t="s">
         <v>290</v>
       </c>
@@ -5278,7 +5299,7 @@
       </c>
       <c r="D133" s="13"/>
     </row>
-    <row r="134" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A134" s="6" t="s">
         <v>292</v>
       </c>
@@ -5290,7 +5311,7 @@
       </c>
       <c r="D134" s="13"/>
     </row>
-    <row r="135" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A135" s="6" t="s">
         <v>294</v>
       </c>
@@ -5302,7 +5323,7 @@
       </c>
       <c r="D135" s="13"/>
     </row>
-    <row r="136" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A136" s="6" t="s">
         <v>296</v>
       </c>
@@ -5314,7 +5335,7 @@
       </c>
       <c r="D136" s="13"/>
     </row>
-    <row r="137" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A137" s="6" t="s">
         <v>298</v>
       </c>
@@ -5326,7 +5347,7 @@
       </c>
       <c r="D137" s="13"/>
     </row>
-    <row r="138" spans="1:4" s="2" customFormat="1" ht="54" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:4" ht="54" x14ac:dyDescent="0.3">
       <c r="A138" s="6" t="s">
         <v>175</v>
       </c>
@@ -5340,7 +5361,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="139" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A139" s="6" t="s">
         <v>300</v>
       </c>
@@ -5352,7 +5373,7 @@
       </c>
       <c r="D139" s="13"/>
     </row>
-    <row r="140" spans="1:4" s="2" customFormat="1" ht="67.5" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:4" ht="67.5" x14ac:dyDescent="0.3">
       <c r="A140" s="6" t="s">
         <v>178</v>
       </c>
@@ -5366,7 +5387,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="141" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A141" s="6" t="s">
         <v>180</v>
       </c>
@@ -5380,7 +5401,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="142" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A142" s="6" t="s">
         <v>183</v>
       </c>
@@ -5394,7 +5415,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="143" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A143" s="6" t="s">
         <v>358</v>
       </c>
@@ -5408,7 +5429,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="144" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A144" s="6" t="s">
         <v>20</v>
       </c>
@@ -5422,7 +5443,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="145" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A145" s="6" t="s">
         <v>416</v>
       </c>
@@ -5436,7 +5457,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="146" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A146" s="6" t="s">
         <v>445</v>
       </c>
@@ -5450,7 +5471,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="147" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A147" s="6" t="s">
         <v>579</v>
       </c>
@@ -5464,7 +5485,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="148" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A148" s="6" t="s">
         <v>581</v>
       </c>
@@ -5478,7 +5499,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="149" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A149" s="6" t="s">
         <v>309</v>
       </c>
@@ -5492,7 +5513,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="150" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A150" s="6" t="s">
         <v>312</v>
       </c>
@@ -5506,7 +5527,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="151" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A151" s="6" t="s">
         <v>360</v>
       </c>
@@ -5518,7 +5539,7 @@
       </c>
       <c r="D151" s="13"/>
     </row>
-    <row r="152" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A152" s="6" t="s">
         <v>315</v>
       </c>
@@ -5530,7 +5551,7 @@
       </c>
       <c r="D152" s="13"/>
     </row>
-    <row r="153" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A153" s="6" t="s">
         <v>317</v>
       </c>
@@ -5542,7 +5563,7 @@
       </c>
       <c r="D153" s="13"/>
     </row>
-    <row r="154" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A154" s="6" t="s">
         <v>418</v>
       </c>
@@ -5556,7 +5577,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="155" spans="1:4" s="2" customFormat="1" ht="54" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:4" ht="54" x14ac:dyDescent="0.3">
       <c r="A155" s="6" t="s">
         <v>188</v>
       </c>
@@ -5570,7 +5591,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:4" s="2" customFormat="1" ht="67.5" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:4" ht="67.5" x14ac:dyDescent="0.3">
       <c r="A156" s="6" t="s">
         <v>189</v>
       </c>
@@ -5584,7 +5605,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="157" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A157" s="6" t="s">
         <v>191</v>
       </c>
@@ -5598,7 +5619,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="158" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A158" s="6" t="s">
         <v>194</v>
       </c>
@@ -5612,7 +5633,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="159" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A159" s="6" t="s">
         <v>375</v>
       </c>
@@ -5622,7 +5643,7 @@
       <c r="C159" s="5"/>
       <c r="D159" s="13"/>
     </row>
-    <row r="160" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A160" s="6" t="s">
         <v>589</v>
       </c>
@@ -5636,7 +5657,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="161" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A161" s="6" t="s">
         <v>197</v>
       </c>
@@ -5648,7 +5669,7 @@
       </c>
       <c r="D161" s="13"/>
     </row>
-    <row r="162" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A162" s="6" t="s">
         <v>201</v>
       </c>
@@ -5662,7 +5683,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="163" spans="1:4" s="2" customFormat="1" ht="81" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:4" ht="81" x14ac:dyDescent="0.3">
       <c r="A163" s="6" t="s">
         <v>591</v>
       </c>
@@ -5676,7 +5697,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="164" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A164" s="6" t="s">
         <v>204</v>
       </c>
@@ -5690,7 +5711,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="165" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A165" s="6" t="s">
         <v>324</v>
       </c>
@@ -5702,7 +5723,7 @@
       </c>
       <c r="D165" s="13"/>
     </row>
-    <row r="166" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A166" s="6" t="s">
         <v>322</v>
       </c>
@@ -5714,7 +5735,7 @@
       </c>
       <c r="D166" s="13"/>
     </row>
-    <row r="167" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A167" s="6" t="s">
         <v>326</v>
       </c>
@@ -5726,7 +5747,7 @@
       </c>
       <c r="D167" s="13"/>
     </row>
-    <row r="168" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A168" s="6" t="s">
         <v>208</v>
       </c>
@@ -5740,7 +5761,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="169" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A169" s="6" t="s">
         <v>209</v>
       </c>
@@ -5754,7 +5775,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="170" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A170" s="6" t="s">
         <v>211</v>
       </c>
@@ -5768,7 +5789,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="171" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A171" s="6" t="s">
         <v>213</v>
       </c>
@@ -5782,7 +5803,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="172" spans="1:4" s="2" customFormat="1" ht="54" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:4" ht="54" x14ac:dyDescent="0.3">
       <c r="A172" s="6" t="s">
         <v>372</v>
       </c>
@@ -5794,7 +5815,7 @@
       </c>
       <c r="D172" s="13"/>
     </row>
-    <row r="173" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A173" s="6" t="s">
         <v>221</v>
       </c>
@@ -5806,7 +5827,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="174" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A174" s="6" t="s">
         <v>219</v>
       </c>
@@ -5818,7 +5839,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="175" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A175" s="6" t="s">
         <v>218</v>
       </c>
@@ -5830,7 +5851,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="176" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A176" s="6" t="s">
         <v>222</v>
       </c>
@@ -5844,7 +5865,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="177" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A177" s="6" t="s">
         <v>224</v>
       </c>
@@ -5858,7 +5879,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="178" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A178" s="6" t="s">
         <v>227</v>
       </c>
@@ -5872,7 +5893,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="179" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A179" s="6" t="s">
         <v>229</v>
       </c>
@@ -5886,7 +5907,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="180" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A180" s="6" t="s">
         <v>231</v>
       </c>
@@ -5900,7 +5921,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="181" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A181" s="6" t="s">
         <v>236</v>
       </c>
@@ -5914,7 +5935,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="182" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A182" s="6" t="s">
         <v>583</v>
       </c>
@@ -5928,7 +5949,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="183" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A183" s="6" t="s">
         <v>594</v>
       </c>
@@ -5942,7 +5963,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="184" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A184" s="6" t="s">
         <v>241</v>
       </c>
@@ -5956,7 +5977,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="185" spans="1:4" s="2" customFormat="1" ht="54" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:4" ht="54" x14ac:dyDescent="0.3">
       <c r="A185" s="6" t="s">
         <v>435</v>
       </c>
@@ -5970,7 +5991,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="186" spans="1:4" s="2" customFormat="1" ht="54" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:4" ht="54" x14ac:dyDescent="0.3">
       <c r="A186" s="6" t="s">
         <v>438</v>
       </c>
@@ -5984,7 +6005,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="187" spans="1:4" s="2" customFormat="1" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
       <c r="A187" s="17" t="s">
         <v>598</v>
       </c>
@@ -5998,7 +6019,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="188" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A188" s="17" t="s">
         <v>599</v>
       </c>
@@ -6006,7 +6027,7 @@
       <c r="C188" s="19"/>
       <c r="D188" s="13"/>
     </row>
-    <row r="189" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A189" s="17" t="s">
         <v>600</v>
       </c>
@@ -6014,7 +6035,7 @@
       <c r="C189" s="19"/>
       <c r="D189" s="13"/>
     </row>
-    <row r="190" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A190" s="20" t="s">
         <v>619</v>
       </c>
@@ -6028,7 +6049,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="191" spans="1:4" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:4" ht="27" x14ac:dyDescent="0.3">
       <c r="A191" s="20" t="s">
         <v>622</v>
       </c>
@@ -6040,6 +6061,20 @@
       </c>
       <c r="D191" s="13" t="s">
         <v>451</v>
+      </c>
+    </row>
+    <row r="192" spans="1:4" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A192" s="20" t="s">
+        <v>631</v>
+      </c>
+      <c r="B192" s="18" t="s">
+        <v>633</v>
+      </c>
+      <c r="C192" s="19" t="s">
+        <v>632</v>
+      </c>
+      <c r="D192" s="13" t="s">
+        <v>634</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
* useCountryIP tenant_config문서에 추가
</commit_message>
<xml_diff>
--- a/docs/config/tbl_tenant_config 정리문서.xlsx
+++ b/docs/config/tbl_tenant_config 정리문서.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DC317\git\ezFlow4Java\docs\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\eGovFrameDev-3.5.1-64bit\workspace\ezFlow4Java\docs\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="635">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="639">
   <si>
     <t>LangPrimary3</t>
   </si>
@@ -3007,6 +3007,23 @@
   </si>
   <si>
     <t>일정등록 공개범위 기본값 설정 여부</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NO</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>useCountryIP</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">메일 발신국가의 국기를 표시할지 여부 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>YES : 사용
+NO : 사용안함</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -3479,7 +3496,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D192"/>
+  <dimension ref="A1:D193"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40.625" style="2" customWidth="1"/>
@@ -6075,6 +6092,20 @@
       </c>
       <c r="D192" s="13" t="s">
         <v>634</v>
+      </c>
+    </row>
+    <row r="193" spans="1:4" ht="27" x14ac:dyDescent="0.3">
+      <c r="A193" s="20" t="s">
+        <v>635</v>
+      </c>
+      <c r="B193" s="18" t="s">
+        <v>636</v>
+      </c>
+      <c r="C193" s="19" t="s">
+        <v>637</v>
+      </c>
+      <c r="D193" s="13" t="s">
+        <v>638</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
일정관리 useScheduleIcs tenant_config 값 추가
</commit_message>
<xml_diff>
--- a/docs/config/tbl_tenant_config 정리문서.xlsx
+++ b/docs/config/tbl_tenant_config 정리문서.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="639">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="641">
   <si>
     <t>LangPrimary3</t>
   </si>
@@ -3028,6 +3028,14 @@
   </si>
   <si>
     <t>NO</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>useScheduleIcs</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>일정관리 ICS파일 가져오기 기능 사용 여부</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -3496,7 +3504,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D193"/>
+  <dimension ref="A1:D194"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40.625" style="2" customWidth="1"/>
@@ -6106,6 +6114,20 @@
       </c>
       <c r="D193" s="13" t="s">
         <v>638</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4" ht="27" x14ac:dyDescent="0.3">
+      <c r="A194" s="20" t="s">
+        <v>639</v>
+      </c>
+      <c r="B194" s="18" t="s">
+        <v>640</v>
+      </c>
+      <c r="C194" s="19" t="s">
+        <v>623</v>
+      </c>
+      <c r="D194" s="13" t="s">
+        <v>448</v>
       </c>
     </row>
   </sheetData>

</xml_diff>